<commit_message>
Move STATUS CENSO para a primeira coluna da planilha modelo
Facilita a visualizacao do andamento; CPF/NOME/TURNO continuam nas
colunas B/C/D que o script le.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MODELO_PLANILHA.xlsx
+++ b/MODELO_PLANILHA.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -446,112 +446,118 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>STATUS CENSO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CPF</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NOME</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TURNO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>DT. INGRESSO</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>CPF</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>NOME</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>TURNO</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DT. NASCIMENTO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PAI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>SEXO</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>COR</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>NATURALIDADE</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>TURMA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>00000000000</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ALUNO DE EXEMPLO (APAGUE ESTA LINHA)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>MATUTINO</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>01/02/2025</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>00000000000</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>ALUNO DE EXEMPLO (APAGUE ESTA LINHA)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>MATUTINO</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>10/05/2008</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>MAE DE EXEMPLO</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>PAI DE EXEMPLO</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>PARDA</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>BRASILIA-DF</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -564,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -581,112 +587,118 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>STATUS CENSO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CPF</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NOME</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TURNO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>DT. INGRESSO</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>CPF</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>NOME</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>TURNO</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DT. NASCIMENTO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PAI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>SEXO</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>COR</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>NATURALIDADE</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>TURMA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>00000000000</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ALUNO DE EXEMPLO (APAGUE ESTA LINHA)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>MATUTINO</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>01/02/2025</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>00000000000</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>ALUNO DE EXEMPLO (APAGUE ESTA LINHA)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>MATUTINO</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>10/05/2008</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>MAE DE EXEMPLO</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>PAI DE EXEMPLO</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>PARDA</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>BRASILIA-DF</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Move STATUS CENSO para a primeira coluna da planilha modelo (#1)
* Move STATUS CENSO para a primeira coluna da planilha modelo

Facilita a visualizacao do andamento; CPF/NOME/TURNO continuam nas
colunas B/C/D que o script le.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>

* Ignora tambem os backups da planilha real (DADOSCENSO*.xlsx)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MODELO_PLANILHA.xlsx
+++ b/MODELO_PLANILHA.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -446,112 +446,118 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>STATUS CENSO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CPF</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NOME</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TURNO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>DT. INGRESSO</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>CPF</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>NOME</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>TURNO</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DT. NASCIMENTO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PAI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>SEXO</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>COR</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>NATURALIDADE</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>TURMA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>00000000000</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ALUNO DE EXEMPLO (APAGUE ESTA LINHA)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>MATUTINO</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>01/02/2025</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>00000000000</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>ALUNO DE EXEMPLO (APAGUE ESTA LINHA)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>MATUTINO</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>10/05/2008</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>MAE DE EXEMPLO</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>PAI DE EXEMPLO</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>PARDA</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>BRASILIA-DF</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -564,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -581,112 +587,118 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>STATUS CENSO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CPF</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NOME</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TURNO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>DT. INGRESSO</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>CPF</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>NOME</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>TURNO</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DT. NASCIMENTO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PAI</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>SEXO</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>COR</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>NATURALIDADE</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>TURMA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>00000000000</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ALUNO DE EXEMPLO (APAGUE ESTA LINHA)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>MATUTINO</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>01/02/2025</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>00000000000</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>ALUNO DE EXEMPLO (APAGUE ESTA LINHA)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>MATUTINO</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>10/05/2008</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>MAE DE EXEMPLO</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>PAI DE EXEMPLO</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>PARDA</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>BRASILIA-DF</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Painel de filtros resiliente e coluna UF de nascimento na planilha
O painel de busca detalhada recolhe sozinho apos re-render do Angular;
agora abre+digita em loop ate os valores persistirem. Nova coluna UF
(apos NATURALIDADE) passa a ser a fonte da UF de nascimento no
cadastro, com fallback para capitais reconhecidas. Modelo e README
atualizados.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MODELO_PLANILHA.xlsx
+++ b/MODELO_PLANILHA.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -501,6 +501,11 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>UF</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>TURMA</t>
         </is>
       </c>
@@ -554,10 +559,15 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>BRASILIA-DF</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+          <t>BRASILIA</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -570,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -642,6 +652,11 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>UF</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>TURMA</t>
         </is>
       </c>
@@ -695,10 +710,15 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>BRASILIA-DF</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+          <t>BRASILIA</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>